<commit_message>
docs(qa): ciclos de prueba, informe Sprint 1-3, E2E de UI y seguridad/carga de la corrida del 16/10
</commit_message>
<xml_diff>
--- a/docs/qa/Plan_de_pruebas_Sprint_1-4.xlsx
+++ b/docs/qa/Plan_de_pruebas_Sprint_1-4.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos y pendientes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Parte A - Manuales'!$A$1:$M$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Parte A - Manuales'!$A$1:$M$212</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pasos TC'!$A$1:$E$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Parte B - Automatizados'!$A$1:$L$449</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defectos y pendientes'!$A$1:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defectos y pendientes'!$A$1:$F$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -538,23 +538,23 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$195,B5)</f>
+        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$212,B5)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B5,'Parte A - Manuales'!$J$2:$J$195,"OK")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B5,'Parte A - Manuales'!$J$2:$J$212,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B5,'Parte A - Manuales'!$J$2:$J$195,"Falla")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B5,'Parte A - Manuales'!$J$2:$J$212,"Falla")</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B5,'Parte A - Manuales'!$J$2:$J$195,"Bloqueado")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B5,'Parte A - Manuales'!$J$2:$J$212,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G5" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B5,'Parte A - Manuales'!$J$2:$J$195,"Pendiente")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B5,'Parte A - Manuales'!$J$2:$J$212,"Pendiente")</f>
         <v/>
       </c>
     </row>
@@ -570,23 +570,23 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$195,B6)</f>
+        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$212,B6)</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B6,'Parte A - Manuales'!$J$2:$J$195,"OK")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B6,'Parte A - Manuales'!$J$2:$J$212,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B6,'Parte A - Manuales'!$J$2:$J$195,"Falla")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B6,'Parte A - Manuales'!$J$2:$J$212,"Falla")</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B6,'Parte A - Manuales'!$J$2:$J$195,"Bloqueado")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B6,'Parte A - Manuales'!$J$2:$J$212,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G6" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B6,'Parte A - Manuales'!$J$2:$J$195,"Pendiente")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B6,'Parte A - Manuales'!$J$2:$J$212,"Pendiente")</f>
         <v/>
       </c>
     </row>
@@ -602,55 +602,55 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$195,B7)</f>
+        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$212,B7)</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B7,'Parte A - Manuales'!$J$2:$J$195,"OK")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B7,'Parte A - Manuales'!$J$2:$J$212,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B7,'Parte A - Manuales'!$J$2:$J$195,"Falla")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B7,'Parte A - Manuales'!$J$2:$J$212,"Falla")</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B7,'Parte A - Manuales'!$J$2:$J$195,"Bloqueado")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B7,'Parte A - Manuales'!$J$2:$J$212,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G7" s="3">
-        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$195,B7,'Parte A - Manuales'!$J$2:$J$195,"Pendiente")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B7,'Parte A - Manuales'!$J$2:$J$212,"Pendiente")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Automatizados (TA)</t>
+          <t>Manuales (TC)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sprint 1-2</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="C8" s="3">
-        <f>COUNTIF('Parte B - Automatizados'!$B$2:$B$449,B8)</f>
+        <f>COUNTIF('Parte A - Manuales'!$B$2:$B$212,B8)</f>
         <v/>
       </c>
       <c r="D8" s="3">
-        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B8,'Parte B - Automatizados'!$J$2:$J$449,"OK")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B8,'Parte A - Manuales'!$J$2:$J$212,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B8,'Parte B - Automatizados'!$J$2:$J$449,"Falla")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B8,'Parte A - Manuales'!$J$2:$J$212,"Falla")</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B8,'Parte B - Automatizados'!$J$2:$J$449,"Bloqueado")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B8,'Parte A - Manuales'!$J$2:$J$212,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G8" s="3">
-        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B8,'Parte B - Automatizados'!$J$2:$J$449,"Pendiente")</f>
+        <f>COUNTIFS('Parte A - Manuales'!$B$2:$B$212,B8,'Parte A - Manuales'!$J$2:$J$212,"Pendiente")</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 1-2</t>
         </is>
       </c>
       <c r="C9" s="3">
@@ -694,7 +694,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C10" s="3">
@@ -719,140 +719,179 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Automatizados (TA)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C11" s="3">
+        <f>COUNTIF('Parte B - Automatizados'!$B$2:$B$449,B11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B11,'Parte B - Automatizados'!$J$2:$J$449,"OK")</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B11,'Parte B - Automatizados'!$J$2:$J$449,"Falla")</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B11,'Parte B - Automatizados'!$J$2:$J$449,"Bloqueado")</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>COUNTIFS('Parte B - Automatizados'!$B$2:$B$449,B11,'Parte B - Automatizados'!$J$2:$J$449,"Pendiente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="4">
-        <f>SUM(C5:C10)</f>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4">
+        <f>SUM(C5:C11)</f>
         <v/>
       </c>
-      <c r="D11" s="4">
-        <f>SUM(D5:D10)</f>
+      <c r="D12" s="4">
+        <f>SUM(D5:D11)</f>
         <v/>
       </c>
-      <c r="E11" s="4">
-        <f>SUM(E5:E10)</f>
+      <c r="E12" s="4">
+        <f>SUM(E5:E11)</f>
         <v/>
       </c>
-      <c r="F11" s="4">
-        <f>SUM(F5:F10)</f>
+      <c r="F12" s="4">
+        <f>SUM(F5:F11)</f>
         <v/>
       </c>
-      <c r="G11" s="4">
-        <f>SUM(G5:G10)</f>
+      <c r="G12" s="4">
+        <f>SUM(G5:G11)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Última ejecución (2026-10-14, rama dev con el trabajo de Sprint 4 integrado)</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Backend: 259 pruebas unitarias y 248 de integración, todas OK (incluye el endpoint de esquema de medicación, SCRUM-232).</t>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Última ejecución (2026-10-16, rama dev + correcciones de QA)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Frontend: 29 archivos / 120 pruebas y build de producción, OK (incluye asistencia y medicación de Sprint 4, que usan datos simulados).</t>
+          <t>Backend: ver cifras de la corrida en el informe (unitarias e integración, todas OK; el 16/10 se agregó un test unitario por el aviso de bloqueo en el 5º intento).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>UI en navegador real (Playwright): 33 de 33 verificaciones OK el 2026-10-09; no se volvió a correr el 2026-10-12 (necesita el stack completo).</t>
+          <t>Frontend: 29 archivos / 122 pruebas y build de producción, OK.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Prueba de humo por rol (Referente, Directora, Escucha, Coordinador): 11 de 15 pantallas OK; las 4 restantes son /inicio (ver Defectos y pendientes).</t>
+          <t>UI en navegador real (Playwright): sprint1-2-ui-flows.mjs, 35 de 35 verificaciones OK tras corregir 6 defectos hallados en la primera pasada (#22 a #27).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>QA manual Sprint 1-2 (TC-01 a TC-40): 40 de 40 OK el 2026-10-06.</t>
+          <t>Matriz rol x pantalla (Referente, Directora, Escucha, Coordinador): permisos correctos en todas las rutas; solo 'Informes' apunta a /inicio (#5).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sprint 4: 48 casos manuales derivados de los criterios de Jira, todos Pendientes. Solo el esquema de medicación (SCRUM-232) tiene backend y tests; asistencia, agenda, stock e historial todavía no.</t>
+          <t>Seguridad y carga (security/api-security-and-load.mjs): 13 verificaciones de seguridad y 4 de carga OK, sin errores bajo 50 usuarios concurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>QA manual Sprint 1-2 (TC-01 a TC-40): 40 de 40 OK; 23 de ellos se re-ejecutaron en navegador real el 2026-10-16.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sprint 4: 48 casos manuales derivados de los criterios de Jira, todos Pendientes (backend sin desarrollar salvo SCRUM-232).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Épicas / historias cubiertas</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Sprint 1-2: EP-01 Fichas de personas · EP-02 Observaciones e historia de vida · EP-03 Cuentas, roles y notificaciones · EP-10 Asistencia · EP-12 Casa de Convivencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Sprint 4: EP-10 Asistencia (SCRUM-54, 55, 56, 57) · Medicación (SCRUM-59, 60, 61, 71, 75)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Sprint 1-2: EP-01 Fichas de personas · EP-02 Observaciones e historia de vida · EP-03 Cuentas, roles y notificaciones · EP-10 Asistencia · EP-12 Casa de Convivencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sprint 4: EP-10 Asistencia (SCRUM-54, 55, 56, 57) · Medicación (SCRUM-59, 60, 61, 71, 75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Sprint 3: EP-04 Calendario general y personal (SCRUM-15, 16, 17) · EP-05 Colaboradores (SCRUM-18, 19) y visitas de la Casa de Convivencia (SCRUM-74)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Hojas</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Parte A - Manuales: un caso por fila con sus pasos; el estado se completa desde la lista desplegable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Pasos TC: los TC del Sprint 1-2 con una fila por paso (#, Paso, Dato, Esperamos).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Parte B - Automatizados: un test xUnit por fila. Sprint 3 deriva su descripción del nombre del test.</t>
+          <t>Parte A - Manuales: un caso por fila con sus pasos; el estado se completa desde la lista desplegable.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
+        <is>
+          <t>Pasos TC: los TC del Sprint 1-2 con una fila por paso (#, Paso, Dato, Esperamos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Parte B - Automatizados: un test xUnit por fila. Sprint 3 deriva su descripción del nombre del test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Defectos y pendientes: hallazgos de la ejecución y decisiones abiertas.</t>
         </is>
@@ -869,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M195"/>
+  <dimension ref="A1:M212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -997,7 +1036,11 @@
 3. Intentar iniciar sesión con las credenciales recién creadas.  →  El sistema informa que la cuenta está "Pendiente de aprobación" y no permite el acceso.</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1005,7 +1048,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
@@ -1013,7 +1056,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr"/>
+      <c r="M2" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Registro desde la UI: la cuenta queda en /auth/pending-approval y un login con esa cuenta vuelve a la pantalla de pendiente.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1058,7 +1105,11 @@
 3. Seleccionar el rol Escucha y confirmar.  →  La cuenta pasa a estado "Activa" con el rol Escucha asignado.</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr"/>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1066,7 +1117,7 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -1074,7 +1125,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Un Referente aprueba la cuenta desde Usuarios &gt; Pendientes eligiendo el rol; desaparece de Pendientes y la cuenta ingresa al dashboard.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -1117,7 +1172,11 @@
           <t>1. Ingresar el correo electrónico y la contraseña, y hacer clic en Entrar.  →  El sistema valida las credenciales y redirige al panel principal según el rol del usuario.</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1125,7 +1184,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
@@ -1133,7 +1192,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr"/>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Con clave incorrecta se muestra 'Correo o contraseña incorrectos.', no se ingresa y se limpia la contraseña.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1178,7 +1241,11 @@
 3. Intentar iniciar sesión nuevamente con la contraseña correcta.  →  El sistema no permite el acceso mientras la cuenta permanezca bloqueada.</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1186,7 +1253,7 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -1194,7 +1261,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>FALLÓ en la primera ejecución en navegador (DEF-22, DEF-23); corregido y re-ejecutado OK. Primera ejecución: el 5º intento respondía 401 sin avisar del bloqueo y, con la clave correcta, el login navegaba a /auth/blocked (ruta inexistente, pantalla en blanco). Tras la corrección: el 5º intento devuelve 403 y muestra 'Alcanzaste el máximo de intentos permitidos: tu cuenta quedó bloqueada por 30 minutos.'; con la clave correcta la cuenta sigue bloqueada.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -1360,7 +1431,11 @@
 2. Intentar iniciar sesión con las credenciales de la cuenta desactivada.  →  El sistema deniega el acceso e informa que la cuenta se encuentra desactivada.</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1368,7 +1443,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -1376,7 +1451,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>FALLÓ en la primera ejecución en navegador (DEF-24); corregido y re-ejecutado OK. Primera ejecución: la cuenta desactivada no ingresaba pero veía 'No pudimos iniciar sesión. Probá de nuevo en unos minutos.'. Tras la corrección muestra 'Tu cuenta está desactivada. Contactá a un Referente para reactivarla.'.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1420,7 +1499,11 @@
 2. Abrir la ficha donde se registró la observación previa.  →  La observación se sigue mostrando en la línea de tiempo con su autor y fecha originales.</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1428,7 +1511,7 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
@@ -1436,7 +1519,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Inactivar desde Usuarios mueve la cuenta a Inactivos; al reactivarla vuelve a ingresar al dashboard.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -1480,7 +1567,11 @@
 2. Iniciar sesión como Referente y revisar el panel de notificaciones.  →  Se muestra una notificación indicando que hay una cuenta pendiente de aprobación.</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1488,7 +1579,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -1496,7 +1587,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M10" s="7" t="inlineStr"/>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Al registrarse una cuenta, el Referente ve la notificación en la campana y el contador de no leídas aumenta.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1601,7 +1696,11 @@
 3. Intentar guardar otra ficha dejando el nombre vacío.  →  El sistema rechaza el guardado e indica que el nombre es obligatorio.</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1609,7 +1708,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -1617,7 +1716,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Alta mínima (nombre, apellido, DNI): la ficha se crea y aparece en el listado y el detalle. Una ficha vacía muestra los obligatorios y un DNI con letras muestra 'El DNI solo puede tener números, sin puntos ni espacios.'.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1661,7 +1764,11 @@
 2. Abrir una ficha.  →  La ficha se visualiza sin opciones de edición.</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1669,7 +1776,7 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -1677,7 +1784,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>FALLÓ en la primera ejecución en navegador (DEF-26); corregido y re-ejecutado OK. Primera ejecución: Escucha veía 'Editar ficha' en el detalle y el ícono de editar en el listado. Tras la corrección no los ve, no ve 'Nueva ficha' y /edit lo redirige a acceso denegado.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1722,7 +1833,11 @@
 3. Buscar un texto sin coincidencias.  →  El sistema muestra una lista vacía, sin error.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1730,7 +1845,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
@@ -1738,7 +1853,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr"/>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Buscar 'jose&lt;n&gt; nunez' encuentra 'José&lt;n&gt; Núñez'; la búsqueda por DNI la encuentra y una búsqueda sin coincidencias no lista fichas.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1782,7 +1901,11 @@
 2. Repetir con una fecha de ingreso futura.  →  El sistema rechaza el guardado con el mismo mensaje.</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1790,7 +1913,7 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -1798,7 +1921,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>FALLÓ en la primera ejecución en navegador (DEF-25); corregido y re-ejecutado OK. Primera ejecución: con fecha futura la UI mostraba el mensaje genérico 'Ocurrió un error al guardar la ficha.'. Tras la corrección muestra el motivo de la API ('...no puede ser futura.') y no guarda.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1843,7 +1970,11 @@
 3. Cambiar de página con un listado de más de una página.  →  La paginación refleja el total real de resultados.</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1851,7 +1982,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
@@ -1859,7 +1990,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. El filtro por DNI del listado se aplica sin errores de API y muestra el filtro activo.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1903,7 +2038,11 @@
 2. Elegir una categoría, escribir el texto y guardar.  →  Se muestra el modal de éxito y la observación aparece en la línea de tiempo con autor y fecha.</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1911,7 +2050,7 @@
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
@@ -1919,7 +2058,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Se registra una observación con categoría (6 disponibles) y aparece en la línea de tiempo con su autor.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1963,7 +2106,11 @@
 2. Filtrar por una categoría.  →  Solo se muestran las observaciones de esa categoría y el conteo coincide.</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1971,7 +2118,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
@@ -1979,7 +2126,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr"/>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Filtrar por categoría deja solo las observaciones de esa categoría y el filtro por autor responde sin errores.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2024,7 +2175,11 @@
 3. Exportar con un filtro sin resultados.  →  El CSV contiene solo el encabezado.</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2032,7 +2187,7 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
@@ -2040,7 +2195,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. 'Exportar informe' descarga observaciones_&lt;id&gt;.csv.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -2144,7 +2303,11 @@
 2. Volver a guardar la misma etapa con otro texto.  →  Se ve el contenido nuevo y el anterior permanece en el historial.</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2152,7 +2315,7 @@
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -2160,7 +2323,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. La historia de vida muestra las 3 etapas y se agrega una entrada en la primera.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2505,7 +2672,11 @@
 2. Intentar la misma acción por API.  →  El sistema responde 403 (CannotActOnSelf).</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr"/>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2513,7 +2684,7 @@
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
@@ -2521,7 +2692,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M27" s="7" t="inlineStr"/>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. En la fila de la propia cuenta, 'Reasignar Rol' e 'Inactivar' están deshabilitados.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2804,7 +2979,11 @@
           <t>1. Ingresar a la pantalla de Login y hacer clic en Entrar sin completar nada.  →  El formulario solicita completar los campos y no se envía ninguna solicitud al servidor.</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2812,7 +2991,7 @@
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr">
@@ -2820,7 +2999,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M32" s="7" t="inlineStr"/>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Login vacío: se muestran 'El correo electrónico es obligatorio.' y 'La contraseña es obligatoria.' y no se envía la petición.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2864,7 +3047,11 @@
 2. Hacer clic en Registrarme.  →  El sistema rechaza el registro (409) e informa que el correo ya está registrado.</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2872,7 +3059,7 @@
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L33" s="7" t="inlineStr">
@@ -2880,7 +3067,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M33" s="7" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Registrar un correo existente muestra 'Ya existe un usuario registrado con ese email.' y permanece en el formulario.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2985,7 +3176,11 @@
 2. Modificar un dato y guardar.  →  El sistema guarda los cambios y los muestra en el perfil de la ficha.</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2993,7 +3188,7 @@
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
@@ -3001,7 +3196,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M35" s="7" t="inlineStr"/>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. La edición carga el nombre guardado y los cambios se guardan y se ven en el detalle.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3165,7 +3364,11 @@
 2. Elegir una categoría, dejar el texto vacío y guardar.  →  El formulario rechaza el guardado y no se crea ninguna observación.</t>
         </is>
       </c>
-      <c r="I38" s="7" t="inlineStr"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3173,7 +3376,7 @@
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
@@ -3181,7 +3384,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M38" s="7" t="inlineStr"/>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. Con el texto vacío el botón Guardar está deshabilitado y el modal sigue abierto.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3225,7 +3432,11 @@
 2. Intentar guardar.  →  No se suma una entrada en blanco al historial de la etapa.</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3233,7 +3444,7 @@
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
@@ -3241,7 +3452,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M39" s="7" t="inlineStr"/>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>FALLÓ en la primera ejecución en navegador (DEF-27); corregido y re-ejecutado OK. Primera ejecución: con solo espacios el botón quedaba habilitado y la API respondía 400. Tras la corrección el botón queda deshabilitado.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3285,7 +3500,11 @@
 2. Observar el contenido principal.  →  El contenido usa todo el ancho disponible de la pantalla.</t>
         </is>
       </c>
-      <c r="I40" s="7" t="inlineStr"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3293,7 +3512,7 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
@@ -3301,7 +3520,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M40" s="7" t="inlineStr"/>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. En 390 px de ancho no hay desborde horizontal en el inicio ni en el listado de fichas.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3345,7 +3568,11 @@
 2. Elegir otra sección del menú.  →  El sistema navega a la sección elegida y el menú lateral se cierra automáticamente.</t>
         </is>
       </c>
-      <c r="I41" s="7" t="inlineStr"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
           <t>OK</t>
@@ -3353,7 +3580,7 @@
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="L41" s="7" t="inlineStr">
@@ -3361,7 +3588,11 @@
           <t>Mateo Pavoni</t>
         </is>
       </c>
-      <c r="M41" s="7" t="inlineStr"/>
+      <c r="M41" s="7" t="inlineStr">
+        <is>
+          <t>OK en navegador real. En pantalla chica el menú se abre con el botón y se oculta al elegir una opción.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -12716,10 +12947,1157 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" s="7" t="inlineStr">
+        <is>
+          <t>TC-195</t>
+        </is>
+      </c>
+      <c r="B196" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C196" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D196" s="7" t="inlineStr">
+        <is>
+          <t>Los endpoints protegidos exigen sesión</t>
+        </is>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>Sin token, la API no entrega datos.</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G196" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H196" s="7" t="inlineStr">
+        <is>
+          <t>1. GET de 7 rutas protegidas (fichas, listado, usuarios, notificaciones, colaboradores, calendarios) sin Authorization  →  Todas responden 401</t>
+        </is>
+      </c>
+      <c r="I196" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J196" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K196" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L196" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M196" s="7" t="inlineStr">
+        <is>
+          <t>Las 7 rutas respondieron 401.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="7" t="inlineStr">
+        <is>
+          <t>TC-196</t>
+        </is>
+      </c>
+      <c r="B197" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C197" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D197" s="7" t="inlineStr">
+        <is>
+          <t>Autorización por rol en la API</t>
+        </is>
+      </c>
+      <c r="E197" s="7" t="inlineStr">
+        <is>
+          <t>Cada rol solo accede a lo que le corresponde.</t>
+        </is>
+      </c>
+      <c r="F197" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G197" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H197" s="7" t="inlineStr">
+        <is>
+          <t>1. Escucha intenta POST api/social-records  →  403
+2. Escucha, Coordinador y Directora piden api/auth/users/active  →  403</t>
+        </is>
+      </c>
+      <c r="I197" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J197" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K197" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L197" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M197" s="7" t="inlineStr">
+        <is>
+          <t>Crear ficha como Escucha: 403. Listar usuarios como Escucha, Coordinador y Directora: 403.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="7" t="inlineStr">
+        <is>
+          <t>TC-197</t>
+        </is>
+      </c>
+      <c r="B198" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C198" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D198" s="7" t="inlineStr">
+        <is>
+          <t>Un token manipulado se rechaza</t>
+        </is>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>Un JWT con el rol alterado, sin firma válida o malformado no da acceso.</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G198" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H198" s="7" t="inlineStr">
+        <is>
+          <t>1. Cambiar el rol del payload a Referente conservando la firma  →  401
+2. Token con alg=none  →  401
+3. Token malformado  →  401</t>
+        </is>
+      </c>
+      <c r="I198" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J198" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K198" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L198" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M198" s="7" t="inlineStr">
+        <is>
+          <t>Firma alterada, alg=none y token malformado: 401 en los tres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="7" t="inlineStr">
+        <is>
+          <t>TC-198</t>
+        </is>
+      </c>
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t>Inyección SQL en la búsqueda</t>
+        </is>
+      </c>
+      <c r="E199" s="7" t="inlineStr">
+        <is>
+          <t>La búsqueda está parametrizada.</t>
+        </is>
+      </c>
+      <c r="F199" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G199" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H199" s="7" t="inlineStr">
+        <is>
+          <t>1. Buscar "' OR 1=1 --" y "'; DROP TABLE Persons; --"  →  Sin error 500 y sin devolver todo el listado</t>
+        </is>
+      </c>
+      <c r="I199" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J199" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K199" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L199" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M199" s="7" t="inlineStr">
+        <is>
+          <t>Sin errores 500; la búsqueda devolvió 4 de 15 fichas por coincidencia de texto (no un OR 1=1) y las tablas siguen intactas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="inlineStr">
+        <is>
+          <t>TC-199</t>
+        </is>
+      </c>
+      <c r="B200" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C200" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D200" s="7" t="inlineStr">
+        <is>
+          <t>El login no revela si el correo existe</t>
+        </is>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>Mismo mensaje para correo inexistente y clave incorrecta.</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G200" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H200" s="7" t="inlineStr">
+        <is>
+          <t>1. Login con correo inexistente  →  401 'Credenciales inválidas.'
+2. Login con correo existente y clave incorrecta  →  Misma respuesta</t>
+        </is>
+      </c>
+      <c r="I200" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J200" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K200" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L200" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M200" s="7" t="inlineStr">
+        <is>
+          <t>Ambas respuestas fueron 401 con el mismo cuerpo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="inlineStr">
+        <is>
+          <t>TC-200</t>
+        </is>
+      </c>
+      <c r="B201" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C201" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t>Política de contraseñas</t>
+        </is>
+      </c>
+      <c r="E201" s="7" t="inlineStr">
+        <is>
+          <t>El registro rechaza contraseñas débiles.</t>
+        </is>
+      </c>
+      <c r="F201" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G201" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H201" s="7" t="inlineStr">
+        <is>
+          <t>1. Registrar con la contraseña '123'  →  400</t>
+        </is>
+      </c>
+      <c r="I201" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J201" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K201" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L201" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M201" s="7" t="inlineStr">
+        <is>
+          <t>Respondió 400.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="7" t="inlineStr">
+        <is>
+          <t>TC-201</t>
+        </is>
+      </c>
+      <c r="B202" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C202" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t>Asignación masiva en el registro</t>
+        </is>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>Enviar role, roleId y status en el registro no otorga privilegios.</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G202" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H202" s="7" t="inlineStr">
+        <is>
+          <t>1. Registrar enviando role=Referente, roleId y status=Active  →  La cuenta queda Pendiente
+2. Intentar loguear  →  403 Pending</t>
+        </is>
+      </c>
+      <c r="I202" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J202" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K202" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L202" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M202" s="7" t="inlineStr">
+        <is>
+          <t>Registro 201 y login 403 con estado Pending: los campos extra se ignoran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="7" t="inlineStr">
+        <is>
+          <t>TC-202</t>
+        </is>
+      </c>
+      <c r="B203" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C203" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t>XSS: la API no cae ante HTML en los datos</t>
+        </is>
+      </c>
+      <c r="E203" s="7" t="inlineStr">
+        <is>
+          <t>Un nombre con HTML no produce errores del servidor.</t>
+        </is>
+      </c>
+      <c r="F203" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G203" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H203" s="7" t="inlineStr">
+        <is>
+          <t>1. Crear una ficha con nombre '&lt;img src=x onerror=...&gt;'  →  Rechazo 4xx o guardado sin error 500</t>
+        </is>
+      </c>
+      <c r="I203" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J203" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K203" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L203" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M203" s="7" t="inlineStr">
+        <is>
+          <t>La API respondió 400 (nombre inválido).</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="7" t="inlineStr">
+        <is>
+          <t>TC-203</t>
+        </is>
+      </c>
+      <c r="B204" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C204" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D204" s="7" t="inlineStr">
+        <is>
+          <t>XSS almacenado en una observación (UI)</t>
+        </is>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>El texto con HTML/script se muestra como texto y no ejecuta código.</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G204" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H204" s="7" t="inlineStr">
+        <is>
+          <t>1. Registrar una observación con &lt;img onerror&gt; y &lt;script&gt;  →  Se muestra el texto literal
+2. Verificar que no se ejecutó código en la página  →  window.__xss no está definido</t>
+        </is>
+      </c>
+      <c r="I204" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/e2e/sprint1-2-ui-flows.mjs</t>
+        </is>
+      </c>
+      <c r="J204" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K204" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L204" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M204" s="7" t="inlineStr">
+        <is>
+          <t>La observación se muestra como texto y no se ejecutó ningún script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="inlineStr">
+        <is>
+          <t>TC-204</t>
+        </is>
+      </c>
+      <c r="B205" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C205" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D205" s="7" t="inlineStr">
+        <is>
+          <t>Cabeceras de seguridad del frontend</t>
+        </is>
+      </c>
+      <c r="E205" s="7" t="inlineStr">
+        <is>
+          <t>El servidor web envía cabeceras defensivas.</t>
+        </is>
+      </c>
+      <c r="F205" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G205" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H205" s="7" t="inlineStr">
+        <is>
+          <t>1. Pedir /auth y revisar cabeceras  →  X-Content-Type-Options, X-Frame-Options, Content-Security-Policy y Referrer-Policy presentes</t>
+        </is>
+      </c>
+      <c r="I205" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J205" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K205" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L205" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M205" s="7" t="inlineStr">
+        <is>
+          <t>Las cuatro cabeceras están presentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="7" t="inlineStr">
+        <is>
+          <t>TC-205</t>
+        </is>
+      </c>
+      <c r="B206" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C206" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D206" s="7" t="inlineStr">
+        <is>
+          <t>La API no expone la versión del servidor</t>
+        </is>
+      </c>
+      <c r="E206" s="7" t="inlineStr">
+        <is>
+          <t>Sin X-Powered-By ni versión en Server.</t>
+        </is>
+      </c>
+      <c r="F206" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G206" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H206" s="7" t="inlineStr">
+        <is>
+          <t>1. Pedir una ruta de la API y revisar cabeceras  →  Sin X-Powered-By; Server sin número de versión</t>
+        </is>
+      </c>
+      <c r="I206" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J206" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K206" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L206" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M206" s="7" t="inlineStr">
+        <is>
+          <t>Server: Kestrel, sin X-Powered-By.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="7" t="inlineStr">
+        <is>
+          <t>TC-206</t>
+        </is>
+      </c>
+      <c r="B207" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C207" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t>Payload de 2 MB y JSON malformado</t>
+        </is>
+      </c>
+      <c r="E207" s="7" t="inlineStr">
+        <is>
+          <t>La API rechaza entradas anómalas sin romperse ni filtrar trazas.</t>
+        </is>
+      </c>
+      <c r="F207" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G207" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H207" s="7" t="inlineStr">
+        <is>
+          <t>1. POST con un nombre de 2 MB  →  4xx
+2. POST con JSON incompleto  →  400 sin stack trace</t>
+        </is>
+      </c>
+      <c r="I207" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J207" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K207" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L207" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M207" s="7" t="inlineStr">
+        <is>
+          <t>2 MB: 400. JSON malformado: 400 sin trazas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="inlineStr">
+        <is>
+          <t>TC-207</t>
+        </is>
+      </c>
+      <c r="B208" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C208" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D208" s="7" t="inlineStr">
+        <is>
+          <t>Ids inexistentes o mal formados</t>
+        </is>
+      </c>
+      <c r="E208" s="7" t="inlineStr">
+        <is>
+          <t>Sin errores 500 ni datos de otros registros.</t>
+        </is>
+      </c>
+      <c r="F208" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G208" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H208" s="7" t="inlineStr">
+        <is>
+          <t>1. GET de una ficha con un GUID inexistente  →  404
+2. GET con un id mal formado ('1;DROP')  →  4xx</t>
+        </is>
+      </c>
+      <c r="I208" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J208" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K208" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L208" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M208" s="7" t="inlineStr">
+        <is>
+          <t>Inexistente: 404. Mal formado: 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="7" t="inlineStr">
+        <is>
+          <t>TC-208</t>
+        </is>
+      </c>
+      <c r="B209" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C209" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D209" s="7" t="inlineStr">
+        <is>
+          <t>Carga: listado de fichas</t>
+        </is>
+      </c>
+      <c r="E209" s="7" t="inlineStr">
+        <is>
+          <t>50 usuarios concurrentes consultando el listado.</t>
+        </is>
+      </c>
+      <c r="F209" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G209" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H209" s="7" t="inlineStr">
+        <is>
+          <t>1. 500 pedidos GET api/social-records/list con 50 en paralelo  →  Sin errores y p95 &lt; 2000 ms</t>
+        </is>
+      </c>
+      <c r="I209" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J209" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K209" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L209" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M209" s="7" t="inlineStr">
+        <is>
+          <t>Listado de fichas: 50 usuarios concurrentes, 500 pedidos, 0 errores, 486.9 pedidos/s, p50 89 ms, p95 195 ms, máximo 318 ms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="7" t="inlineStr">
+        <is>
+          <t>TC-209</t>
+        </is>
+      </c>
+      <c r="B210" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C210" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D210" s="7" t="inlineStr">
+        <is>
+          <t>Carga: notificaciones</t>
+        </is>
+      </c>
+      <c r="E210" s="7" t="inlineStr">
+        <is>
+          <t>50 usuarios concurrentes consultando notificaciones.</t>
+        </is>
+      </c>
+      <c r="F210" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G210" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H210" s="7" t="inlineStr">
+        <is>
+          <t>1. 500 pedidos GET api/notifications con 50 en paralelo  →  Sin errores y p95 &lt; 2000 ms</t>
+        </is>
+      </c>
+      <c r="I210" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J210" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K210" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L210" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M210" s="7" t="inlineStr">
+        <is>
+          <t>Notificaciones: 50 usuarios concurrentes, 500 pedidos, 0 errores, 756.9 pedidos/s, p50 62 ms, p95 101 ms, máximo 161 ms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="7" t="inlineStr">
+        <is>
+          <t>TC-210</t>
+        </is>
+      </c>
+      <c r="B211" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C211" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D211" s="7" t="inlineStr">
+        <is>
+          <t>Carga: calendario general</t>
+        </is>
+      </c>
+      <c r="E211" s="7" t="inlineStr">
+        <is>
+          <t>30 usuarios concurrentes consultando el calendario.</t>
+        </is>
+      </c>
+      <c r="F211" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G211" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H211" s="7" t="inlineStr">
+        <is>
+          <t>1. 300 pedidos GET api/general-calendar-events con 30 en paralelo  →  Sin errores y p95 &lt; 2000 ms</t>
+        </is>
+      </c>
+      <c r="I211" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J211" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K211" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L211" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M211" s="7" t="inlineStr">
+        <is>
+          <t>Calendario general: 30 usuarios concurrentes, 300 pedidos, 0 errores, 545.1 pedidos/s, p50 49 ms, p95 89 ms, máximo 101 ms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="7" t="inlineStr">
+        <is>
+          <t>TC-211</t>
+        </is>
+      </c>
+      <c r="B212" s="7" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C212" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad y rendimiento</t>
+        </is>
+      </c>
+      <c r="D212" s="7" t="inlineStr">
+        <is>
+          <t>Carga: inicio de sesión</t>
+        </is>
+      </c>
+      <c r="E212" s="7" t="inlineStr">
+        <is>
+          <t>20 usuarios concurrentes iniciando sesión (bcrypt).</t>
+        </is>
+      </c>
+      <c r="F212" s="7" t="inlineStr">
+        <is>
+          <t>Stack local levantado (docker compose en backend/); usuarios de prueba *@test.com.</t>
+        </is>
+      </c>
+      <c r="G212" s="7" t="inlineStr">
+        <is>
+          <t>RNF seguridad / rendimiento</t>
+        </is>
+      </c>
+      <c r="H212" s="7" t="inlineStr">
+        <is>
+          <t>1. 100 pedidos POST api/auth/login con 20 en paralelo  →  Sin errores y p95 &lt; 3000 ms</t>
+        </is>
+      </c>
+      <c r="I212" s="7" t="inlineStr">
+        <is>
+          <t>docs/qa/security/api-security-and-load.mjs</t>
+        </is>
+      </c>
+      <c r="J212" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K212" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="L212" s="7" t="inlineStr">
+        <is>
+          <t>Mateo Pavoni</t>
+        </is>
+      </c>
+      <c r="M212" s="7" t="inlineStr">
+        <is>
+          <t>Login: 20 usuarios concurrentes, 100 pedidos, 0 errores, 11.6 pedidos/s, p50 1674 ms, p95 2781 ms, máximo 3110 ms.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M195"/>
+  <autoFilter ref="A1:M212"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J195" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,OK,Falla,Bloqueado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -42606,7 +43984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -42780,7 +44158,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Los ítems del menú Inicio, Asistencia, Medicación e Informes apuntan a /inicio, una ruta sin pantalla (página vacía). Está en main.</t>
+          <t>Los ítems Inicio, Asistencia y Medicación ya funcionan; solo 'Informes' apunta a /inicio, una ruta sin pantalla (página vacía). Verificado en navegador con los 4 roles el 2026-10-16.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -43279,8 +44657,248 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Defecto</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Cuenta bloqueada: el login navegaba a /auth/blocked, una ruta que no existe, y dejaba la pantalla en blanco sin ningún mensaje.</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-84 / 94 (frontend)</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Corregido en dev</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>login.component.ts ahora muestra el aviso de bloqueo en el propio formulario. Re-ejecutado OK en navegador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Defecto</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>El quinto intento fallido de login bloqueaba la cuenta pero respondía 401 'Credenciales inválidas': no informaba el bloqueo hasta el sexto intento.</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-84 (AuthService)</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Corregido en dev</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>AuthService.LoginAsync devuelve AccountLocked en el intento que dispara el bloqueo; test unitario nuevo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Defecto</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Una cuenta desactivada que intentaba ingresar veía 'No pudimos iniciar sesión. Probá de nuevo en unos minutos.' (el frontend no mapeaba el estado Inactive de la API).</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-20 (frontend)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Corregido en dev</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>AuthService.mapError distingue Inactive y Rejected; mensajes específicos y tests nuevos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Defecto</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Al guardar una ficha con fecha futura la UI mostraba el mensaje genérico 'Ocurrió un error al guardar la ficha.' aunque la API devolvía 'La fecha de ingreso no puede ser futura.'.</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-5 (frontend)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Corregido en dev</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Las pantallas de alta y edición usan extractApiError y muestran el motivo de validación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Defecto</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>El rol Escucha veía el botón 'Editar ficha' en el detalle y el ícono de editar en el listado (la ruta /edit sí lo rechazaba con acceso denegado).</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-13 / 64 (frontend)</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Corregido en dev</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Ambos controles se muestran solo con el permiso fichas.edit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Defecto</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Una observación con solo espacios habilitaba el botón Guardar; el backend la rechazaba con 400.</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-9 (frontend)</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Corregido en dev</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>El formulario valida el largo mínimo sobre el texto recortado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Pregunta abierta</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>La API acepta crear dos fichas con el mismo DNI (201 y 201). Los colaboradores sí rechazan DNI duplicado (409).</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-5 / EP-01</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Confirmar si el DNI debe ser único en fichas antes de agregar la regla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Pregunta abierta</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>La API permite crear fichas al Coordinador de Casa de Convivencia (POST api/social-records), pero la UI le deniega /fichas/crear.</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>SCRUM-13 / 64</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Se suma a la pregunta #20 sobre los permisos del Coordinador.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F22"/>
+  <autoFilter ref="A1:F30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>